<commit_message>
refactor: zamień dane mogące pochodzić z firmy na fikcyjne
Przewoźnicy GLS/GEIS -> PACZKI/PALETY, firmowe kody stref (92xx, WCxx,
LABO, PPAP, CRET, RETV, BROK, ZP92) -> fikcyjne, magazyn DLT i tabela
Power BI Stock_oraz_DLT -> ZEW, odbiorca PHARMO -> DOMEX, numery dostaw
8178xxxx -> 8000xxxx, branża medyczna -> ceramika. Model GlsPackingEntry ->
ParcelPackingEntry (migracja huctl 0006, dane zostają), trasa
gls_packing_report -> parcel_packing_report, env GLS_ZONE_CODES ->
PARCEL_ZONE_CODES. Usunięte szablony: lokalizacje_uklad (realne stosy z
eksportu EWM) i wzor_import_ukraina (usunięty moduł).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESHqYcHmR7ZBD8zM8mFg5s
</commit_message>
<xml_diff>
--- a/excel_templates/GROOVE_ankieta_proces_kontroli.xlsx
+++ b/excel_templates/GROOVE_ankieta_proces_kontroli.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Instrukcja" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="GEIS paletowa kraj" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="PALETY paletowa kraj" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Export paletowy" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="GLS paczkowa" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PACZKI paczkowa" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="BUS" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
@@ -693,7 +693,7 @@
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Główny obszar (GEIS kraj / Export / GLS / BUS):</t>
+          <t>Główny obszar (PALETY kraj / Export / PACZKI / BUS):</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Obszar: Wysyłka paletowa krajowa (GEIS)</t>
+          <t>Obszar: Wysyłka paletowa krajowa (PALETY)</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Obszar: Wysyłka paletowa eksportowa (poza GEIS)</t>
+          <t>Obszar: Wysyłka paletowa eksportowa (poza PALETY)</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Obszar: Wysyłka paczkowa (GLS)</t>
+          <t>Obszar: Wysyłka paczkowa (PACZKI)</t>
         </is>
       </c>
     </row>

</xml_diff>